<commit_message>
all readme files are updated
</commit_message>
<xml_diff>
--- a/mutationResults/AalborgProblem/WithTrack/Comparison of SPEA2 with SPEA2_DK for each generation (on average).xlsx
+++ b/mutationResults/AalborgProblem/WithTrack/Comparison of SPEA2 with SPEA2_DK for each generation (on average).xlsx
@@ -897,11 +897,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="122174656"/>
-        <c:axId val="122171912"/>
+        <c:axId val="383769088"/>
+        <c:axId val="383762032"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="122174656"/>
+        <c:axId val="383769088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -922,31 +922,6 @@
           </c:spPr>
         </c:majorGridlines>
         <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="it-IT"/>
-                  <a:t>Generation</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
           <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
@@ -1014,12 +989,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="122171912"/>
+        <c:crossAx val="383762032"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="122171912"/>
+        <c:axId val="383762032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1039,6 +1014,37 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1076,7 +1082,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="122174656"/>
+        <c:crossAx val="383769088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1089,7 +1095,7 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="t"/>
+      <c:legendPos val="r"/>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -1962,11 +1968,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="317534584"/>
-        <c:axId val="317530272"/>
+        <c:axId val="383762816"/>
+        <c:axId val="383757720"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="317534584"/>
+        <c:axId val="383762816"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2079,12 +2085,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317530272"/>
+        <c:crossAx val="383757720"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="317530272"/>
+        <c:axId val="383757720"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2141,7 +2147,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317534584"/>
+        <c:crossAx val="383762816"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2153,38 +2159,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:layout/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="it-IT"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -3027,11 +3001,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="317532232"/>
-        <c:axId val="317538504"/>
+        <c:axId val="383759288"/>
+        <c:axId val="383756936"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="317532232"/>
+        <c:axId val="383759288"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3144,12 +3118,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317538504"/>
+        <c:crossAx val="383756936"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="317538504"/>
+        <c:axId val="383756936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.65000000000000013"/>
@@ -3207,7 +3181,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317532232"/>
+        <c:crossAx val="383759288"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3219,38 +3193,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:layout/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="it-IT"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -4093,11 +4035,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="317538896"/>
-        <c:axId val="317539288"/>
+        <c:axId val="383759680"/>
+        <c:axId val="383763208"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="317538896"/>
+        <c:axId val="383759680"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,12 +4152,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317539288"/>
+        <c:crossAx val="383763208"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="317539288"/>
+        <c:axId val="383763208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4272,7 +4214,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317538896"/>
+        <c:crossAx val="383759680"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4284,38 +4226,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:layout/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="it-IT"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -5158,11 +5068,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="317534976"/>
-        <c:axId val="317533408"/>
+        <c:axId val="383760072"/>
+        <c:axId val="383766344"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="317534976"/>
+        <c:axId val="383760072"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5275,12 +5185,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317533408"/>
+        <c:crossAx val="383766344"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="317533408"/>
+        <c:axId val="383766344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5337,7 +5247,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="317534976"/>
+        <c:crossAx val="383760072"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5349,38 +5259,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:layout/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="it-IT"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>

</xml_diff>